<commit_message>
fresh save and export of PDF and BOM
</commit_message>
<xml_diff>
--- a/bici-pcb/Project Outputs for bici-pcb/bici-pcb.xlsx
+++ b/bici-pcb/Project Outputs for bici-pcb/bici-pcb.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\truth\OneDrive\Desktop\ACADEMICS\ENGN1650\engn1650-bici-pcb\bici-pcb\Project Outputs for bici-pcb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{85043DCA-A5A7-4381-AF0C-03A3EC3029D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F518039B-6261-4E0E-8FA6-BC69C86C5050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2808" yWindow="2808" windowWidth="17280" windowHeight="10134" xr2:uid="{D5D973EB-1224-46A1-97CA-BD7A8676D3D4}"/>
+    <workbookView xWindow="2808" yWindow="2808" windowWidth="17280" windowHeight="10134" xr2:uid="{9E3A43A7-1431-4810-AE2F-B9B64BF6C1AC}"/>
   </bookViews>
   <sheets>
     <sheet name="bici-pcb" sheetId="1" r:id="rId1"/>
@@ -377,6 +377,21 @@
     <t>0</t>
   </si>
   <si>
+    <t>ERJ-3EKF1002V</t>
+  </si>
+  <si>
+    <t>RES SMD 10K OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>R101, R102, R103, R104, R215, R216, R301, R303, R402, R404</t>
+  </si>
+  <si>
+    <t>667-ERJ-3EKF1002V</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
     <t>ERJ-3EKF1200V</t>
   </si>
   <si>
@@ -390,21 +405,6 @@
   </si>
   <si>
     <t>120</t>
-  </si>
-  <si>
-    <t>ERJ-3EKF1002V</t>
-  </si>
-  <si>
-    <t>RES SMD 10K OHM 1% 1/10W 0603</t>
-  </si>
-  <si>
-    <t>R215, R216, R301, R303, R402, R404</t>
-  </si>
-  <si>
-    <t>667-ERJ-3EKF1002V</t>
-  </si>
-  <si>
-    <t>10k</t>
   </si>
   <si>
     <t>ERJ-P06J110V</t>
@@ -938,7 +938,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{359627E5-9883-4B82-BC93-CDBE6EE2AB2A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C50E00CE-F706-4030-9514-773453EEF678}">
   <dimension ref="A1:J29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -1544,7 +1544,7 @@
         <v>115</v>
       </c>
       <c r="D20" s="1">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>94</v>
@@ -1553,7 +1553,7 @@
         <v>113</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>116</v>
@@ -1576,7 +1576,7 @@
         <v>120</v>
       </c>
       <c r="D21" s="1">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>94</v>
@@ -1585,7 +1585,7 @@
         <v>118</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>121</v>

</xml_diff>